<commit_message>
added Measurement Core's projections from May 2025
</commit_message>
<xml_diff>
--- a/inst/extdata/biospecimen_collection_for_biostore_calculations.xlsx
+++ b/inst/extdata/biospecimen_collection_for_biostore_calculations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/meghanshilts/r_code/biostoreCapacity/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{995CADB5-E65F-6943-AF5C-360FC78F0C81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4AD932A-BA41-C04B-A9B7-B651771271D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9400" yWindow="7220" windowWidth="23960" windowHeight="17380" xr2:uid="{F08E2CC1-CD3C-F641-B418-A953A5DB15A9}"/>
+    <workbookView xWindow="320" yWindow="3420" windowWidth="23960" windowHeight="17380" xr2:uid="{F08E2CC1-CD3C-F641-B418-A953A5DB15A9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="62">
   <si>
     <t>whole_blood_maternal</t>
   </si>
@@ -195,9 +195,6 @@
   </si>
   <si>
     <t>set to 1 because this wasn't officially changed. We couldn't remove this collection until we added 11-17 blood spot (which needed IRB approval) so i think it was decided this would change in 2026 to add 11-17 blood spot and remove 11-17 whole blood in 2026</t>
-  </si>
-  <si>
-    <t>set to 1 because this wasn't officially changed. We couldn't remove this collection until we added 11-17 blood spot (which needed IRB approval) so i think it was decided this would change in 2026 to add 11-17 blood spot and remove 11-17 whole blood in 202</t>
   </si>
   <si>
     <t>y_2025_proportion</t>
@@ -308,13 +305,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -932,40 +930,40 @@
         <v>31</v>
       </c>
       <c r="Q1" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="R1" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="T1" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="U1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="V1" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="V1" s="2" t="s">
-        <v>59</v>
       </c>
       <c r="W1" s="2" t="s">
         <v>43</v>
       </c>
       <c r="X1" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="Y1" s="2" t="s">
         <v>45</v>
       </c>
       <c r="Z1" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AA1" s="2" t="s">
         <v>46</v>
       </c>
       <c r="AB1" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AC1" s="3" t="s">
         <v>50</v>
@@ -1043,27 +1041,27 @@
         <v>1</v>
       </c>
       <c r="X2" s="1">
-        <v>0.5</v>
+        <v>0.42</v>
       </c>
       <c r="Y2" s="1">
         <v>1</v>
       </c>
       <c r="Z2" s="1">
-        <v>0.5</v>
+        <v>0.69</v>
       </c>
       <c r="AA2" s="1">
         <v>1</v>
       </c>
       <c r="AB2" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="AC2" t="s">
+        <v>0.19</v>
+      </c>
+      <c r="AC2" s="6" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A3" t="str">
-        <f t="shared" ref="A3:A28" si="0">B3&amp;"_"&amp;E3&amp;"_"&amp;H3&amp;"_"&amp;J3</f>
+        <f>B3&amp;"_"&amp;E3&amp;"_"&amp;H3&amp;"_"&amp;J3</f>
         <v>breastmilk_1ml_0_5_months_specialized</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -1133,34 +1131,34 @@
         <v>1</v>
       </c>
       <c r="X3" s="1">
-        <v>0.5</v>
+        <v>0.42</v>
       </c>
       <c r="Y3" s="1">
         <v>1</v>
       </c>
       <c r="Z3" s="1">
-        <v>0.5</v>
+        <v>0.69</v>
       </c>
       <c r="AA3" s="1">
         <v>1</v>
       </c>
       <c r="AB3" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="AC3" t="s">
+        <v>0.19</v>
+      </c>
+      <c r="AC3" s="6" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A4" t="str">
-        <f t="shared" si="0"/>
-        <v>cord_blood_1.9ml_perinatal_core</v>
+        <f>B4&amp;"_"&amp;E4&amp;"_"&amp;H4&amp;"_"&amp;J4</f>
+        <v>urine_diaper_1.9ml_12_23_months_specialized</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>17</v>
@@ -1169,19 +1167,19 @@
         <v>13</v>
       </c>
       <c r="F4" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G4" s="1">
-        <v>1</v>
+        <v>0.67</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="I4" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K4" s="1">
         <v>1</v>
@@ -1219,77 +1217,77 @@
       <c r="V4" s="1">
         <v>1</v>
       </c>
-      <c r="W4" s="1" t="s">
-        <v>44</v>
+      <c r="W4" s="1">
+        <v>0</v>
       </c>
       <c r="X4" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="Y4" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="Z4" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="AA4" s="1" t="s">
-        <v>44</v>
+      <c r="Y4" s="1">
+        <v>1</v>
+      </c>
+      <c r="Z4" s="1">
+        <v>0.69</v>
+      </c>
+      <c r="AA4" s="1">
+        <v>0</v>
       </c>
       <c r="AB4" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="AC4" t="s">
+      <c r="AC4" s="6" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A5" t="str">
-        <f t="shared" si="0"/>
-        <v>cord_blood_1ml_perinatal_core</v>
+        <f>B5&amp;"_"&amp;E5&amp;"_"&amp;H5&amp;"_"&amp;J5</f>
+        <v>whole_blood_child_1.9ml_11_17_years_specialized</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>1</v>
+        <v>38</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>17</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F5" s="1">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G5" s="1">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="I5" s="1">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K5" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L5" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M5" s="1">
         <v>1</v>
       </c>
       <c r="N5" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O5" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P5" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q5" s="1">
         <v>0.25</v>
@@ -1309,77 +1307,77 @@
       <c r="V5" s="1">
         <v>1</v>
       </c>
-      <c r="W5" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="X5" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="Y5" s="1" t="s">
-        <v>44</v>
+      <c r="W5" s="1">
+        <v>1</v>
+      </c>
+      <c r="X5" s="1">
+        <v>0.42</v>
+      </c>
+      <c r="Y5" s="1">
+        <v>0</v>
       </c>
       <c r="Z5" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="AA5" s="1" t="s">
-        <v>44</v>
+      <c r="AA5" s="1">
+        <v>0</v>
       </c>
       <c r="AB5" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="AC5" t="s">
+      <c r="AC5" s="6" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A6" t="str">
-        <f t="shared" si="0"/>
-        <v>placenta_1.9ml_perinatal_core</v>
+        <f>B6&amp;"_"&amp;E6&amp;"_"&amp;H6&amp;"_"&amp;J6</f>
+        <v>whole_blood_child_1ml_11_17_years_specialized</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F6" s="1">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G6" s="1">
         <v>0.9</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="I6" s="1">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K6" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L6" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M6" s="1">
         <v>1</v>
       </c>
       <c r="N6" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O6" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P6" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q6" s="1">
         <v>0.25</v>
@@ -1399,77 +1397,77 @@
       <c r="V6" s="1">
         <v>1</v>
       </c>
-      <c r="W6" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="X6" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="Y6" s="1" t="s">
-        <v>44</v>
+      <c r="W6" s="1">
+        <v>1</v>
+      </c>
+      <c r="X6" s="1">
+        <v>0.42</v>
+      </c>
+      <c r="Y6" s="1">
+        <v>0</v>
       </c>
       <c r="Z6" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="AA6" s="1" t="s">
-        <v>44</v>
+      <c r="AA6" s="1">
+        <v>0</v>
       </c>
       <c r="AB6" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="AC6" t="s">
+      <c r="AC6" s="6" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A7" t="str">
-        <f t="shared" si="0"/>
-        <v>urine_cup_maternal_1.9ml_preg_early_core</v>
+        <f>B7&amp;"_"&amp;E7&amp;"_"&amp;H7&amp;"_"&amp;J7</f>
+        <v>whole_blood_child_1.9ml_6_10_years_specialized</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>13</v>
       </c>
       <c r="F7" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G7" s="1">
         <v>1</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="I7" s="1">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K7" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L7" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M7" s="1">
         <v>1</v>
       </c>
       <c r="N7" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O7" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P7" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q7" s="1">
         <v>0.25</v>
@@ -1489,77 +1487,77 @@
       <c r="V7" s="1">
         <v>1</v>
       </c>
-      <c r="W7" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="X7" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="Y7" s="1" t="s">
-        <v>44</v>
+      <c r="W7" s="1">
+        <v>1</v>
+      </c>
+      <c r="X7" s="1">
+        <v>0.42</v>
+      </c>
+      <c r="Y7" s="1">
+        <v>0</v>
       </c>
       <c r="Z7" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="AA7" s="1" t="s">
-        <v>44</v>
+      <c r="AA7" s="1">
+        <v>0</v>
       </c>
       <c r="AB7" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="AC7" t="s">
+      <c r="AC7" s="6" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A8" t="str">
-        <f t="shared" si="0"/>
-        <v>urine_cup_maternal_1.9ml_preg_third_tri_core</v>
+        <f>B8&amp;"_"&amp;E8&amp;"_"&amp;H8&amp;"_"&amp;J8</f>
+        <v>whole_blood_child_1ml_6_10_years_specialized</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F8" s="1">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G8" s="1">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="I8" s="1">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K8" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L8" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M8" s="1">
         <v>1</v>
       </c>
       <c r="N8" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O8" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P8" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q8" s="1">
         <v>0.25</v>
@@ -1579,31 +1577,31 @@
       <c r="V8" s="1">
         <v>1</v>
       </c>
-      <c r="W8" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="X8" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="Y8" s="1" t="s">
-        <v>44</v>
+      <c r="W8" s="1">
+        <v>1</v>
+      </c>
+      <c r="X8" s="1">
+        <v>0.42</v>
+      </c>
+      <c r="Y8" s="1">
+        <v>0</v>
       </c>
       <c r="Z8" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="AA8" s="1" t="s">
-        <v>44</v>
+      <c r="AA8" s="1">
+        <v>0</v>
       </c>
       <c r="AB8" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="AC8" t="s">
+      <c r="AC8" s="6" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A9" t="str">
-        <f t="shared" si="0"/>
+        <f>B9&amp;"_"&amp;E9&amp;"_"&amp;H9&amp;"_"&amp;J9</f>
         <v>urine_diaper_1.9ml_0_5_months_core</v>
       </c>
       <c r="B9" s="1" t="s">
@@ -1693,17 +1691,17 @@
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A10" t="str">
-        <f t="shared" si="0"/>
-        <v>urine_cup_current_partner_1.9ml_6_11_months_preconception</v>
+        <f>B10&amp;"_"&amp;E10&amp;"_"&amp;H10&amp;"_"&amp;J10</f>
+        <v>urine_cup_child_1.9ml_11_17_years_core</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>37</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>13</v>
@@ -1715,31 +1713,31 @@
         <v>1</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="I10" s="1">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="K10" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L10" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M10" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N10" s="1">
         <v>1</v>
       </c>
       <c r="O10" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P10" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q10" s="1">
         <v>0.25</v>
@@ -1778,58 +1776,58 @@
         <v>44</v>
       </c>
       <c r="AC10" s="4" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A11" t="str">
-        <f t="shared" si="0"/>
-        <v>urine_cup_maternal_1.9ml_6_11_months_preconception</v>
+        <f>B11&amp;"_"&amp;E11&amp;"_"&amp;H11&amp;"_"&amp;J11</f>
+        <v>whole_blood_child_1.9ml_11_17_years_core</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>13</v>
       </c>
       <c r="F11" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G11" s="1">
         <v>1</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="I11" s="1">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="K11" s="1">
         <v>1</v>
       </c>
       <c r="L11" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M11" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N11" s="1">
         <v>1</v>
       </c>
       <c r="O11" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P11" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q11" s="1">
         <v>0.25</v>
@@ -1868,58 +1866,58 @@
         <v>44</v>
       </c>
       <c r="AC11" s="5" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A12" t="str">
-        <f t="shared" si="0"/>
-        <v>urine_diaper_1.9ml_12_23_months_specialized</v>
+        <f>B12&amp;"_"&amp;E12&amp;"_"&amp;H12&amp;"_"&amp;J12</f>
+        <v>whole_blood_child_1ml_11_17_years_core</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>17</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F12" s="1">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G12" s="1">
-        <v>0.67</v>
+        <v>0.9</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="I12" s="1">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K12" s="1">
         <v>1</v>
       </c>
       <c r="L12" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M12" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N12" s="1">
         <v>1</v>
       </c>
       <c r="O12" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P12" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q12" s="1">
         <v>0.25</v>
@@ -1939,31 +1937,31 @@
       <c r="V12" s="1">
         <v>1</v>
       </c>
-      <c r="W12" s="1">
-        <v>0</v>
+      <c r="W12" s="1" t="s">
+        <v>44</v>
       </c>
       <c r="X12" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="Y12" s="1">
-        <v>1</v>
-      </c>
-      <c r="Z12" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="AA12" s="1">
-        <v>0</v>
+      <c r="Y12" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z12" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA12" s="1" t="s">
+        <v>44</v>
       </c>
       <c r="AB12" s="1" t="s">
         <v>44</v>
       </c>
       <c r="AC12" s="5" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A13" t="str">
-        <f t="shared" si="0"/>
+        <f>B13&amp;"_"&amp;E13&amp;"_"&amp;H13&amp;"_"&amp;J13</f>
         <v>urine_cup_maternal_1.9ml_24_35_months_preconception</v>
       </c>
       <c r="B13" s="1" t="s">
@@ -2053,7 +2051,7 @@
     </row>
     <row r="14" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A14" t="str">
-        <f t="shared" si="0"/>
+        <f>B14&amp;"_"&amp;E14&amp;"_"&amp;H14&amp;"_"&amp;J14</f>
         <v>urine_hat_1.9ml_3_5_years_core</v>
       </c>
       <c r="B14" s="1" t="s">
@@ -2143,7 +2141,7 @@
     </row>
     <row r="15" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A15" t="str">
-        <f t="shared" si="0"/>
+        <f>B15&amp;"_"&amp;E15&amp;"_"&amp;H15&amp;"_"&amp;J15</f>
         <v>urine_hat_1.9ml_6_10_years_core</v>
       </c>
       <c r="B15" s="1" t="s">
@@ -2233,14 +2231,14 @@
     </row>
     <row r="16" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A16" t="str">
-        <f t="shared" si="0"/>
-        <v>urine_cup_child_1.9ml_11_17_years_core</v>
+        <f>B16&amp;"_"&amp;E16&amp;"_"&amp;H16&amp;"_"&amp;J16</f>
+        <v>whole_blood_child_1.9ml_6_10_years_core</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>17</v>
@@ -2249,16 +2247,16 @@
         <v>13</v>
       </c>
       <c r="F16" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G16" s="1">
         <v>1</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I16" s="1">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J16" s="1" t="s">
         <v>22</v>
@@ -2323,32 +2321,32 @@
     </row>
     <row r="17" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A17" t="str">
-        <f t="shared" si="0"/>
-        <v>whole_blood_maternal_1.9ml_preg_early_core</v>
+        <f>B17&amp;"_"&amp;E17&amp;"_"&amp;H17&amp;"_"&amp;J17</f>
+        <v>whole_blood_child_1ml_6_10_years_core</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>38</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F17" s="1">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G17" s="1">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="I17" s="1">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="J17" s="1" t="s">
         <v>22</v>
@@ -2357,19 +2355,19 @@
         <v>1</v>
       </c>
       <c r="L17" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M17" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N17" s="1">
         <v>1</v>
       </c>
       <c r="O17" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P17" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q17" s="1">
         <v>0.25</v>
@@ -2413,38 +2411,38 @@
     </row>
     <row r="18" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A18" t="str">
-        <f t="shared" si="0"/>
-        <v>whole_blood_maternal_1.9ml_preg_third_tri_core</v>
+        <f>B18&amp;"_"&amp;E18&amp;"_"&amp;H18&amp;"_"&amp;J18</f>
+        <v>urine_cup_current_partner_1.9ml_6_11_months_preconception</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>13</v>
       </c>
       <c r="F18" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G18" s="1">
         <v>1</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="I18" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="K18" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L18" s="1">
         <v>1</v>
@@ -2498,58 +2496,58 @@
         <v>44</v>
       </c>
       <c r="AC18" s="5" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A19" t="str">
-        <f t="shared" si="0"/>
-        <v>whole_blood_child_1.9ml_6_10_years_specialized</v>
+        <f>B19&amp;"_"&amp;E19&amp;"_"&amp;H19&amp;"_"&amp;J19</f>
+        <v>urine_cup_maternal_1.9ml_6_11_months_preconception</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>13</v>
       </c>
       <c r="F19" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G19" s="1">
         <v>1</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="I19" s="1">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="K19" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L19" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M19" s="1">
         <v>1</v>
       </c>
       <c r="N19" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O19" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P19" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q19" s="1">
         <v>0.25</v>
@@ -2569,20 +2567,20 @@
       <c r="V19" s="1">
         <v>1</v>
       </c>
-      <c r="W19" s="1">
-        <v>1</v>
-      </c>
-      <c r="X19" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="Y19" s="1">
-        <v>0</v>
+      <c r="W19" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="X19" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y19" s="1" t="s">
+        <v>44</v>
       </c>
       <c r="Z19" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="AA19" s="1">
-        <v>0</v>
+      <c r="AA19" s="1" t="s">
+        <v>44</v>
       </c>
       <c r="AB19" s="1" t="s">
         <v>44</v>
@@ -2593,14 +2591,14 @@
     </row>
     <row r="20" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A20" t="str">
-        <f t="shared" si="0"/>
-        <v>whole_blood_child_1.9ml_6_10_years_core</v>
+        <f>B20&amp;"_"&amp;E20&amp;"_"&amp;H20&amp;"_"&amp;J20</f>
+        <v>cord_blood_1.9ml_perinatal_core</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>17</v>
@@ -2615,10 +2613,10 @@
         <v>1</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="I20" s="1">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="J20" s="1" t="s">
         <v>22</v>
@@ -2627,19 +2625,19 @@
         <v>1</v>
       </c>
       <c r="L20" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M20" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N20" s="1">
         <v>1</v>
       </c>
       <c r="O20" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P20" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q20" s="1">
         <v>0.25</v>
@@ -2683,53 +2681,53 @@
     </row>
     <row r="21" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A21" t="str">
-        <f t="shared" si="0"/>
-        <v>whole_blood_child_1.9ml_11_17_years_specialized</v>
+        <f>B21&amp;"_"&amp;E21&amp;"_"&amp;H21&amp;"_"&amp;J21</f>
+        <v>cord_blood_1ml_perinatal_core</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>17</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F21" s="1">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G21" s="1">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="I21" s="1">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K21" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L21" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M21" s="1">
         <v>1</v>
       </c>
       <c r="N21" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O21" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P21" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q21" s="1">
         <v>0.25</v>
@@ -2749,20 +2747,20 @@
       <c r="V21" s="1">
         <v>1</v>
       </c>
-      <c r="W21" s="1">
-        <v>1</v>
-      </c>
-      <c r="X21" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="Y21" s="1">
-        <v>0</v>
+      <c r="W21" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="X21" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y21" s="1" t="s">
+        <v>44</v>
       </c>
       <c r="Z21" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="AA21" s="1">
-        <v>0</v>
+      <c r="AA21" s="1" t="s">
+        <v>44</v>
       </c>
       <c r="AB21" s="1" t="s">
         <v>44</v>
@@ -2773,32 +2771,32 @@
     </row>
     <row r="22" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A22" t="str">
-        <f t="shared" si="0"/>
-        <v>whole_blood_child_1.9ml_11_17_years_core</v>
+        <f>B22&amp;"_"&amp;E22&amp;"_"&amp;H22&amp;"_"&amp;J22</f>
+        <v>placenta_1.9ml_perinatal_core</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>38</v>
+        <v>9</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>13</v>
       </c>
       <c r="F22" s="1">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="G22" s="1">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="I22" s="1">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="J22" s="1" t="s">
         <v>22</v>
@@ -2807,19 +2805,19 @@
         <v>1</v>
       </c>
       <c r="L22" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M22" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N22" s="1">
         <v>1</v>
       </c>
       <c r="O22" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P22" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q22" s="1">
         <v>0.25</v>
@@ -2858,31 +2856,31 @@
         <v>44</v>
       </c>
       <c r="AC22" s="4" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
     </row>
     <row r="23" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A23" t="str">
-        <f t="shared" si="0"/>
-        <v>whole_blood_maternal_1ml_preg_early_core</v>
+        <f>B23&amp;"_"&amp;E23&amp;"_"&amp;H23&amp;"_"&amp;J23</f>
+        <v>urine_cup_maternal_1.9ml_preg_early_core</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>16</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F23" s="1">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G23" s="1">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="H23" s="1" t="s">
         <v>24</v>
@@ -2953,8 +2951,8 @@
     </row>
     <row r="24" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A24" t="str">
-        <f t="shared" si="0"/>
-        <v>whole_blood_maternal_1ml_preg_third_tri_core</v>
+        <f>B24&amp;"_"&amp;E24&amp;"_"&amp;H24&amp;"_"&amp;J24</f>
+        <v>whole_blood_maternal_1.9ml_preg_early_core</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>0</v>
@@ -2966,19 +2964,19 @@
         <v>16</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F24" s="1">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G24" s="1">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I24" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J24" s="1" t="s">
         <v>22</v>
@@ -3043,17 +3041,17 @@
     </row>
     <row r="25" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A25" t="str">
-        <f t="shared" si="0"/>
-        <v>whole_blood_child_1ml_6_10_years_specialized</v>
+        <f>B25&amp;"_"&amp;E25&amp;"_"&amp;H25&amp;"_"&amp;J25</f>
+        <v>whole_blood_maternal_1ml_preg_early_core</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>38</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>12</v>
@@ -3065,31 +3063,31 @@
         <v>0.9</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="I25" s="1">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K25" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L25" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M25" s="1">
         <v>1</v>
       </c>
       <c r="N25" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O25" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P25" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q25" s="1">
         <v>0.25</v>
@@ -3109,20 +3107,20 @@
       <c r="V25" s="1">
         <v>1</v>
       </c>
-      <c r="W25" s="1">
-        <v>1</v>
-      </c>
-      <c r="X25" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="Y25" s="1">
-        <v>0</v>
+      <c r="W25" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="X25" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y25" s="1" t="s">
+        <v>44</v>
       </c>
       <c r="Z25" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="AA25" s="1">
-        <v>0</v>
+      <c r="AA25" s="1" t="s">
+        <v>44</v>
       </c>
       <c r="AB25" s="1" t="s">
         <v>44</v>
@@ -3133,32 +3131,32 @@
     </row>
     <row r="26" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A26" t="str">
-        <f t="shared" si="0"/>
-        <v>whole_blood_child_1ml_6_10_years_core</v>
+        <f>B26&amp;"_"&amp;E26&amp;"_"&amp;H26&amp;"_"&amp;J26</f>
+        <v>urine_cup_maternal_1.9ml_preg_third_tri_core</v>
       </c>
       <c r="B26" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F26" s="1">
+        <v>3</v>
+      </c>
+      <c r="G26" s="1">
+        <v>1</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="I26" s="1">
         <v>2</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F26" s="1">
-        <v>10</v>
-      </c>
-      <c r="G26" s="1">
-        <v>0.9</v>
-      </c>
-      <c r="H26" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="I26" s="1">
-        <v>10</v>
       </c>
       <c r="J26" s="1" t="s">
         <v>22</v>
@@ -3167,19 +3165,19 @@
         <v>1</v>
       </c>
       <c r="L26" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M26" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N26" s="1">
         <v>1</v>
       </c>
       <c r="O26" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P26" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q26" s="1">
         <v>0.25</v>
@@ -3223,53 +3221,53 @@
     </row>
     <row r="27" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A27" t="str">
-        <f t="shared" si="0"/>
-        <v>whole_blood_child_1ml_11_17_years_specialized</v>
+        <f>B27&amp;"_"&amp;E27&amp;"_"&amp;H27&amp;"_"&amp;J27</f>
+        <v>whole_blood_maternal_1.9ml_preg_third_tri_core</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>38</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F27" s="1">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G27" s="1">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="I27" s="1">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K27" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L27" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M27" s="1">
         <v>1</v>
       </c>
       <c r="N27" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O27" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P27" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q27" s="1">
         <v>0.25</v>
@@ -3289,20 +3287,20 @@
       <c r="V27" s="1">
         <v>1</v>
       </c>
-      <c r="W27" s="1">
-        <v>1</v>
-      </c>
-      <c r="X27" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="Y27" s="1">
-        <v>0</v>
+      <c r="W27" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="X27" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y27" s="1" t="s">
+        <v>44</v>
       </c>
       <c r="Z27" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="AA27" s="1">
-        <v>0</v>
+      <c r="AA27" s="1" t="s">
+        <v>44</v>
       </c>
       <c r="AB27" s="1" t="s">
         <v>44</v>
@@ -3313,17 +3311,17 @@
     </row>
     <row r="28" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A28" t="str">
-        <f t="shared" si="0"/>
-        <v>whole_blood_child_1ml_11_17_years_core</v>
+        <f>B28&amp;"_"&amp;E28&amp;"_"&amp;H28&amp;"_"&amp;J28</f>
+        <v>whole_blood_maternal_1ml_preg_third_tri_core</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>38</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>12</v>
@@ -3335,10 +3333,10 @@
         <v>0.9</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="I28" s="1">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="J28" s="1" t="s">
         <v>22</v>
@@ -3347,19 +3345,19 @@
         <v>1</v>
       </c>
       <c r="L28" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M28" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N28" s="1">
         <v>1</v>
       </c>
       <c r="O28" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P28" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q28" s="1">
         <v>0.25</v>
@@ -3398,12 +3396,12 @@
         <v>44</v>
       </c>
       <c r="AC28" s="4" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:AB28">
-    <sortCondition ref="C1:C28"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AC28">
+    <sortCondition ref="AB1:AB28"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="C1:D1048576">
@@ -3489,7 +3487,7 @@
       <formula>LEFT(K1,LEN("0"))="0"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W1:AB1048576 AC10:AC28">
+  <conditionalFormatting sqref="AC10:AC28 W1:AB1048576">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="NA">
       <formula>NOT(ISERROR(SEARCH("NA",W1)))</formula>
     </cfRule>

</xml_diff>

<commit_message>
merge PTF kit projections with tubes per kit
</commit_message>
<xml_diff>
--- a/inst/extdata/biospecimen_collection_for_biostore_calculations.xlsx
+++ b/inst/extdata/biospecimen_collection_for_biostore_calculations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/meghanshilts/r_code/biostoreCapacity/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BED1C25C-FE4C-B640-8F9A-269508A168AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{981AA16A-4A5B-FA48-8569-CA1539CF3009}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1840" yWindow="2500" windowWidth="29180" windowHeight="17380" xr2:uid="{F08E2CC1-CD3C-F641-B418-A953A5DB15A9}"/>
+    <workbookView xWindow="1460" yWindow="3160" windowWidth="29180" windowHeight="17380" xr2:uid="{F08E2CC1-CD3C-F641-B418-A953A5DB15A9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="75">
   <si>
     <t>whole_blood_maternal</t>
   </si>
@@ -222,6 +222,45 @@
   </si>
   <si>
     <t>coll_y_2030_proportion</t>
+  </si>
+  <si>
+    <t>specimen_clean</t>
+  </si>
+  <si>
+    <t>maternal_breastmilk_specialized</t>
+  </si>
+  <si>
+    <t>child_urine_diaper_specialized</t>
+  </si>
+  <si>
+    <t>child_urine_diaper_core</t>
+  </si>
+  <si>
+    <t>child_urine_hat_core</t>
+  </si>
+  <si>
+    <t>child_cord_blood_core</t>
+  </si>
+  <si>
+    <t>maternal_placenta_core</t>
+  </si>
+  <si>
+    <t>child_whole_blood_specialized</t>
+  </si>
+  <si>
+    <t>child_urine_cup_core</t>
+  </si>
+  <si>
+    <t>child_whole_blood_core</t>
+  </si>
+  <si>
+    <t>maternal_urine_cup_core</t>
+  </si>
+  <si>
+    <t>maternal_whole_blood_core</t>
+  </si>
+  <si>
+    <t>partner_urine_cup_core</t>
   </si>
 </sst>
 </file>
@@ -863,162 +902,166 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26DF0A69-7549-AB48-B708-1E2A20EA2643}">
-  <dimension ref="A1:AD28"/>
+  <dimension ref="A1:AE28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="40.5" customWidth="1"/>
     <col min="3" max="3" width="23.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="26.33203125" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="17" width="6.83203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="15.6640625" customWidth="1"/>
-    <col min="24" max="24" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="26.6640625" customWidth="1"/>
-    <col min="26" max="26" width="20" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="29.1640625" customWidth="1"/>
-    <col min="28" max="28" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="27.33203125" customWidth="1"/>
+    <col min="4" max="4" width="43.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="26.33203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="18" width="6.83203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="24" width="15.6640625" customWidth="1"/>
+    <col min="25" max="25" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="26.6640625" customWidth="1"/>
+    <col min="27" max="27" width="20" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="29.1640625" customWidth="1"/>
+    <col min="29" max="29" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="27.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>43</v>
       </c>
       <c r="B1" s="3" t="str">
-        <f>_xlfn.CONCAT(I1,"_",E1)</f>
+        <f>_xlfn.CONCAT(J1,"_",F1)</f>
         <v>visit_participant</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="T1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="U1" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="V1" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="W1" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="X1" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="Y1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="AA1" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AB1" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AC1" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AD1" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="AD1" s="3" t="s">
+      <c r="AE1" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A2" t="str">
-        <f t="shared" ref="A2:A28" si="0">C2&amp;"_"&amp;F2&amp;"_"&amp;I2&amp;"_"&amp;K2</f>
+        <f t="shared" ref="A2:A28" si="0">C2&amp;"_"&amp;G2&amp;"_"&amp;J2&amp;"_"&amp;L2</f>
         <v>breastmilk_1.9ml_0_5_months_specialized</v>
       </c>
       <c r="B2" s="6" t="str">
-        <f t="shared" ref="B2:B28" si="1">_xlfn.CONCAT(I2,"_",E2)</f>
+        <f t="shared" ref="B2:B28" si="1">_xlfn.CONCAT(J2,"_",F2)</f>
         <v>0_5_months_maternal</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="1">
+      <c r="H2" s="1">
         <v>8</v>
       </c>
-      <c r="H2" s="1">
-        <v>1</v>
-      </c>
-      <c r="I2" s="1" t="s">
+      <c r="I2" s="1">
+        <v>1</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J2" s="1">
+      <c r="K2" s="1">
         <v>4</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="L2" s="1">
-        <v>1</v>
-      </c>
       <c r="M2" s="1">
         <v>1</v>
       </c>
@@ -1035,11 +1078,11 @@
         <v>1</v>
       </c>
       <c r="R2" s="1">
+        <v>1</v>
+      </c>
+      <c r="S2" s="1">
         <v>0.25</v>
       </c>
-      <c r="S2" s="1">
-        <v>1</v>
-      </c>
       <c r="T2" s="1">
         <v>1</v>
       </c>
@@ -1056,25 +1099,28 @@
         <v>1</v>
       </c>
       <c r="Y2" s="1">
+        <v>1</v>
+      </c>
+      <c r="Z2" s="1">
         <v>0.42</v>
       </c>
-      <c r="Z2" s="1">
-        <v>1</v>
-      </c>
       <c r="AA2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AB2" s="1">
         <v>0.69</v>
       </c>
-      <c r="AB2" s="1">
-        <v>1</v>
-      </c>
       <c r="AC2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AD2" s="1">
         <v>0.19</v>
       </c>
-      <c r="AD2" t="s">
+      <c r="AE2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A3" t="str">
         <f t="shared" si="0"/>
         <v>breastmilk_1ml_0_5_months_specialized</v>
@@ -1087,32 +1133,32 @@
         <v>3</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="1">
+      <c r="H3" s="1">
         <v>10</v>
       </c>
-      <c r="H3" s="1">
+      <c r="I3" s="1">
         <v>0.5</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J3" s="1">
+      <c r="K3" s="1">
         <v>4</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="L3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="L3" s="1">
-        <v>1</v>
-      </c>
       <c r="M3" s="1">
         <v>1</v>
       </c>
@@ -1129,11 +1175,11 @@
         <v>1</v>
       </c>
       <c r="R3" s="1">
+        <v>1</v>
+      </c>
+      <c r="S3" s="1">
         <v>0.25</v>
       </c>
-      <c r="S3" s="1">
-        <v>1</v>
-      </c>
       <c r="T3" s="1">
         <v>1</v>
       </c>
@@ -1150,25 +1196,28 @@
         <v>1</v>
       </c>
       <c r="Y3" s="1">
+        <v>1</v>
+      </c>
+      <c r="Z3" s="1">
         <v>0.42</v>
       </c>
-      <c r="Z3" s="1">
-        <v>1</v>
-      </c>
       <c r="AA3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AB3" s="1">
         <v>0.69</v>
       </c>
-      <c r="AB3" s="1">
-        <v>1</v>
-      </c>
       <c r="AC3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AD3" s="1">
         <v>0.19</v>
       </c>
-      <c r="AD3" t="s">
+      <c r="AE3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A4" t="str">
         <f t="shared" si="0"/>
         <v>urine_diaper_1.9ml_12_23_months_specialized</v>
@@ -1181,32 +1230,32 @@
         <v>4</v>
       </c>
       <c r="D4" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="1">
+      <c r="H4" s="1">
         <v>3</v>
       </c>
-      <c r="H4" s="1">
+      <c r="I4" s="1">
         <v>0.67</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="J4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="J4" s="1">
+      <c r="K4" s="1">
         <v>7</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="L4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="L4" s="1">
-        <v>1</v>
-      </c>
       <c r="M4" s="1">
         <v>1</v>
       </c>
@@ -1223,11 +1272,11 @@
         <v>1</v>
       </c>
       <c r="R4" s="1">
+        <v>1</v>
+      </c>
+      <c r="S4" s="1">
         <v>0.25</v>
       </c>
-      <c r="S4" s="1">
-        <v>1</v>
-      </c>
       <c r="T4" s="1">
         <v>1</v>
       </c>
@@ -1241,28 +1290,31 @@
         <v>1</v>
       </c>
       <c r="X4" s="1">
-        <v>0</v>
-      </c>
-      <c r="Y4" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="Z4" s="1">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="Y4" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="1" t="s">
+        <v>38</v>
       </c>
       <c r="AA4" s="1">
+        <v>1</v>
+      </c>
+      <c r="AB4" s="1">
         <v>0.69</v>
       </c>
-      <c r="AB4" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC4" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="AD4" t="s">
+      <c r="AC4" s="1">
+        <v>0</v>
+      </c>
+      <c r="AD4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A5" t="str">
         <f t="shared" si="0"/>
         <v>whole_blood_child_1.9ml_11_17_years_specialized</v>
@@ -1275,40 +1327,40 @@
         <v>2</v>
       </c>
       <c r="D5" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="1">
+      <c r="H5" s="1">
         <v>6</v>
       </c>
-      <c r="H5" s="1">
-        <v>1</v>
-      </c>
-      <c r="I5" s="1" t="s">
+      <c r="I5" s="1">
+        <v>1</v>
+      </c>
+      <c r="J5" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="J5" s="1">
+      <c r="K5" s="1">
         <v>11</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="L5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="L5" s="1">
-        <v>0</v>
-      </c>
       <c r="M5" s="1">
         <v>0</v>
       </c>
       <c r="N5" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O5" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P5" s="1">
         <v>0</v>
@@ -1317,11 +1369,11 @@
         <v>0</v>
       </c>
       <c r="R5" s="1">
+        <v>0</v>
+      </c>
+      <c r="S5" s="1">
         <v>0.25</v>
       </c>
-      <c r="S5" s="1">
-        <v>1</v>
-      </c>
       <c r="T5" s="1">
         <v>1</v>
       </c>
@@ -1338,25 +1390,28 @@
         <v>1</v>
       </c>
       <c r="Y5" s="1">
+        <v>1</v>
+      </c>
+      <c r="Z5" s="1">
         <v>0.42</v>
       </c>
-      <c r="Z5" s="1">
-        <v>0</v>
-      </c>
-      <c r="AA5" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="AB5" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC5" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="AD5" t="s">
+      <c r="AA5" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AC5" s="1">
+        <v>0</v>
+      </c>
+      <c r="AD5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A6" t="str">
         <f t="shared" si="0"/>
         <v>whole_blood_child_1ml_11_17_years_specialized</v>
@@ -1369,40 +1424,40 @@
         <v>2</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="1">
+      <c r="H6" s="1">
         <v>10</v>
       </c>
-      <c r="H6" s="1">
+      <c r="I6" s="1">
         <v>0.9</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="J6" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="J6" s="1">
+      <c r="K6" s="1">
         <v>11</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="L6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="L6" s="1">
-        <v>0</v>
-      </c>
       <c r="M6" s="1">
         <v>0</v>
       </c>
       <c r="N6" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O6" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P6" s="1">
         <v>0</v>
@@ -1411,11 +1466,11 @@
         <v>0</v>
       </c>
       <c r="R6" s="1">
+        <v>0</v>
+      </c>
+      <c r="S6" s="1">
         <v>0.25</v>
       </c>
-      <c r="S6" s="1">
-        <v>1</v>
-      </c>
       <c r="T6" s="1">
         <v>1</v>
       </c>
@@ -1432,25 +1487,28 @@
         <v>1</v>
       </c>
       <c r="Y6" s="1">
+        <v>1</v>
+      </c>
+      <c r="Z6" s="1">
         <v>0.42</v>
       </c>
-      <c r="Z6" s="1">
-        <v>0</v>
-      </c>
-      <c r="AA6" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="AB6" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC6" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="AD6" t="s">
+      <c r="AA6" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB6" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AC6" s="1">
+        <v>0</v>
+      </c>
+      <c r="AD6" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE6" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A7" t="str">
         <f t="shared" si="0"/>
         <v>whole_blood_child_1.9ml_6_10_years_specialized</v>
@@ -1463,40 +1521,40 @@
         <v>2</v>
       </c>
       <c r="D7" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="1">
+      <c r="H7" s="1">
         <v>6</v>
       </c>
-      <c r="H7" s="1">
-        <v>1</v>
-      </c>
-      <c r="I7" s="1" t="s">
+      <c r="I7" s="1">
+        <v>1</v>
+      </c>
+      <c r="J7" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="J7" s="1">
+      <c r="K7" s="1">
         <v>10</v>
       </c>
-      <c r="K7" s="1" t="s">
+      <c r="L7" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="L7" s="1">
-        <v>0</v>
-      </c>
       <c r="M7" s="1">
         <v>0</v>
       </c>
       <c r="N7" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O7" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P7" s="1">
         <v>0</v>
@@ -1505,11 +1563,11 @@
         <v>0</v>
       </c>
       <c r="R7" s="1">
+        <v>0</v>
+      </c>
+      <c r="S7" s="1">
         <v>0.25</v>
       </c>
-      <c r="S7" s="1">
-        <v>1</v>
-      </c>
       <c r="T7" s="1">
         <v>1</v>
       </c>
@@ -1526,25 +1584,28 @@
         <v>1</v>
       </c>
       <c r="Y7" s="1">
+        <v>1</v>
+      </c>
+      <c r="Z7" s="1">
         <v>0.42</v>
       </c>
-      <c r="Z7" s="1">
-        <v>0</v>
-      </c>
-      <c r="AA7" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="AB7" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC7" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="AD7" t="s">
+      <c r="AA7" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB7" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AC7" s="1">
+        <v>0</v>
+      </c>
+      <c r="AD7" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE7" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A8" t="str">
         <f t="shared" si="0"/>
         <v>whole_blood_child_1ml_6_10_years_specialized</v>
@@ -1557,40 +1618,40 @@
         <v>2</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="1">
+      <c r="H8" s="1">
         <v>10</v>
       </c>
-      <c r="H8" s="1">
+      <c r="I8" s="1">
         <v>0.9</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="J8" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="J8" s="1">
+      <c r="K8" s="1">
         <v>10</v>
       </c>
-      <c r="K8" s="1" t="s">
+      <c r="L8" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="L8" s="1">
-        <v>0</v>
-      </c>
       <c r="M8" s="1">
         <v>0</v>
       </c>
       <c r="N8" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O8" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P8" s="1">
         <v>0</v>
@@ -1599,11 +1660,11 @@
         <v>0</v>
       </c>
       <c r="R8" s="1">
+        <v>0</v>
+      </c>
+      <c r="S8" s="1">
         <v>0.25</v>
       </c>
-      <c r="S8" s="1">
-        <v>1</v>
-      </c>
       <c r="T8" s="1">
         <v>1</v>
       </c>
@@ -1620,25 +1681,28 @@
         <v>1</v>
       </c>
       <c r="Y8" s="1">
+        <v>1</v>
+      </c>
+      <c r="Z8" s="1">
         <v>0.42</v>
       </c>
-      <c r="Z8" s="1">
-        <v>0</v>
-      </c>
-      <c r="AA8" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="AB8" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC8" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="AD8" t="s">
+      <c r="AA8" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB8" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AC8" s="1">
+        <v>0</v>
+      </c>
+      <c r="AD8" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE8" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A9" t="str">
         <f t="shared" si="0"/>
         <v>urine_diaper_1.9ml_0_5_months_core</v>
@@ -1651,32 +1715,32 @@
         <v>4</v>
       </c>
       <c r="D9" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="1">
+      <c r="H9" s="1">
         <v>3</v>
       </c>
-      <c r="H9" s="1">
+      <c r="I9" s="1">
         <v>0.67</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="J9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J9" s="1">
+      <c r="K9" s="1">
         <v>4</v>
       </c>
-      <c r="K9" s="1" t="s">
+      <c r="L9" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="L9" s="1">
-        <v>1</v>
-      </c>
       <c r="M9" s="1">
         <v>1</v>
       </c>
@@ -1693,11 +1757,11 @@
         <v>1</v>
       </c>
       <c r="R9" s="1">
+        <v>1</v>
+      </c>
+      <c r="S9" s="1">
         <v>0.25</v>
       </c>
-      <c r="S9" s="1">
-        <v>1</v>
-      </c>
       <c r="T9" s="1">
         <v>1</v>
       </c>
@@ -1710,8 +1774,8 @@
       <c r="W9" s="1">
         <v>1</v>
       </c>
-      <c r="X9" s="1" t="s">
-        <v>38</v>
+      <c r="X9" s="1">
+        <v>1</v>
       </c>
       <c r="Y9" s="1" t="s">
         <v>38</v>
@@ -1728,11 +1792,14 @@
       <c r="AC9" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AD9" t="s">
+      <c r="AD9" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE9" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A10" t="str">
         <f t="shared" si="0"/>
         <v>urine_cup_child_1.9ml_11_17_years_core</v>
@@ -1745,53 +1812,53 @@
         <v>8</v>
       </c>
       <c r="D10" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="F10" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G10" s="1">
+      <c r="H10" s="1">
         <v>3</v>
       </c>
-      <c r="H10" s="1">
-        <v>1</v>
-      </c>
-      <c r="I10" s="1" t="s">
+      <c r="I10" s="1">
+        <v>1</v>
+      </c>
+      <c r="J10" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="J10" s="1">
+      <c r="K10" s="1">
         <v>11</v>
       </c>
-      <c r="K10" s="1" t="s">
+      <c r="L10" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="L10" s="1">
-        <v>1</v>
-      </c>
       <c r="M10" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N10" s="1">
         <v>0</v>
       </c>
       <c r="O10" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P10" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q10" s="1">
         <v>0</v>
       </c>
       <c r="R10" s="1">
+        <v>0</v>
+      </c>
+      <c r="S10" s="1">
         <v>0.25</v>
       </c>
-      <c r="S10" s="1">
-        <v>1</v>
-      </c>
       <c r="T10" s="1">
         <v>1</v>
       </c>
@@ -1804,8 +1871,8 @@
       <c r="W10" s="1">
         <v>1</v>
       </c>
-      <c r="X10" s="1" t="s">
-        <v>38</v>
+      <c r="X10" s="1">
+        <v>1</v>
       </c>
       <c r="Y10" s="1" t="s">
         <v>38</v>
@@ -1822,11 +1889,14 @@
       <c r="AC10" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AD10" s="4" t="s">
+      <c r="AD10" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE10" s="4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A11" t="str">
         <f t="shared" si="0"/>
         <v>whole_blood_child_1.9ml_11_17_years_core</v>
@@ -1839,53 +1909,53 @@
         <v>2</v>
       </c>
       <c r="D11" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="F11" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="1">
+      <c r="H11" s="1">
         <v>6</v>
       </c>
-      <c r="H11" s="1">
-        <v>1</v>
-      </c>
-      <c r="I11" s="1" t="s">
+      <c r="I11" s="1">
+        <v>1</v>
+      </c>
+      <c r="J11" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="J11" s="1">
+      <c r="K11" s="1">
         <v>11</v>
       </c>
-      <c r="K11" s="1" t="s">
+      <c r="L11" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="L11" s="1">
-        <v>1</v>
-      </c>
       <c r="M11" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N11" s="1">
         <v>0</v>
       </c>
       <c r="O11" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P11" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q11" s="1">
         <v>0</v>
       </c>
       <c r="R11" s="1">
+        <v>0</v>
+      </c>
+      <c r="S11" s="1">
         <v>0.25</v>
       </c>
-      <c r="S11" s="1">
-        <v>1</v>
-      </c>
       <c r="T11" s="1">
         <v>1</v>
       </c>
@@ -1898,8 +1968,8 @@
       <c r="W11" s="1">
         <v>1</v>
       </c>
-      <c r="X11" s="1" t="s">
-        <v>38</v>
+      <c r="X11" s="1">
+        <v>1</v>
       </c>
       <c r="Y11" s="1" t="s">
         <v>38</v>
@@ -1916,11 +1986,14 @@
       <c r="AC11" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AD11" s="5" t="s">
+      <c r="AD11" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE11" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A12" t="str">
         <f t="shared" si="0"/>
         <v>whole_blood_child_1ml_11_17_years_core</v>
@@ -1933,53 +2006,53 @@
         <v>2</v>
       </c>
       <c r="D12" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="F12" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G12" s="1">
+      <c r="H12" s="1">
         <v>10</v>
       </c>
-      <c r="H12" s="1">
+      <c r="I12" s="1">
         <v>0.9</v>
       </c>
-      <c r="I12" s="1" t="s">
+      <c r="J12" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="J12" s="1">
+      <c r="K12" s="1">
         <v>11</v>
       </c>
-      <c r="K12" s="1" t="s">
+      <c r="L12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="L12" s="1">
-        <v>1</v>
-      </c>
       <c r="M12" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N12" s="1">
         <v>0</v>
       </c>
       <c r="O12" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P12" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q12" s="1">
         <v>0</v>
       </c>
       <c r="R12" s="1">
+        <v>0</v>
+      </c>
+      <c r="S12" s="1">
         <v>0.25</v>
       </c>
-      <c r="S12" s="1">
-        <v>1</v>
-      </c>
       <c r="T12" s="1">
         <v>1</v>
       </c>
@@ -1992,8 +2065,8 @@
       <c r="W12" s="1">
         <v>1</v>
       </c>
-      <c r="X12" s="1" t="s">
-        <v>38</v>
+      <c r="X12" s="1">
+        <v>1</v>
       </c>
       <c r="Y12" s="1" t="s">
         <v>38</v>
@@ -2010,11 +2083,14 @@
       <c r="AC12" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AD12" s="5" t="s">
+      <c r="AD12" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE12" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A13" t="str">
         <f t="shared" si="0"/>
         <v>urine_cup_maternal_1.9ml_24_35_months_preconception</v>
@@ -2027,34 +2103,34 @@
         <v>5</v>
       </c>
       <c r="D13" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="F13" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G13" s="1">
+      <c r="H13" s="1">
         <v>3</v>
       </c>
-      <c r="H13" s="1">
-        <v>1</v>
-      </c>
-      <c r="I13" s="1" t="s">
+      <c r="I13" s="1">
+        <v>1</v>
+      </c>
+      <c r="J13" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="J13" s="1">
+      <c r="K13" s="1">
         <v>8</v>
       </c>
-      <c r="K13" s="1" t="s">
+      <c r="L13" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="L13" s="1">
-        <v>0</v>
-      </c>
       <c r="M13" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N13" s="1">
         <v>1</v>
@@ -2069,11 +2145,11 @@
         <v>1</v>
       </c>
       <c r="R13" s="1">
+        <v>1</v>
+      </c>
+      <c r="S13" s="1">
         <v>0.25</v>
       </c>
-      <c r="S13" s="1">
-        <v>1</v>
-      </c>
       <c r="T13" s="1">
         <v>1</v>
       </c>
@@ -2086,8 +2162,8 @@
       <c r="W13" s="1">
         <v>1</v>
       </c>
-      <c r="X13" s="1" t="s">
-        <v>38</v>
+      <c r="X13" s="1">
+        <v>1</v>
       </c>
       <c r="Y13" s="1" t="s">
         <v>38</v>
@@ -2104,11 +2180,14 @@
       <c r="AC13" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AD13" s="4" t="s">
+      <c r="AD13" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE13" s="4" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A14" t="str">
         <f t="shared" si="0"/>
         <v>urine_hat_1.9ml_3_5_years_core</v>
@@ -2121,53 +2200,53 @@
         <v>7</v>
       </c>
       <c r="D14" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E14" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="F14" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G14" s="1">
+      <c r="H14" s="1">
         <v>3</v>
       </c>
-      <c r="H14" s="1">
-        <v>1</v>
-      </c>
-      <c r="I14" s="1" t="s">
+      <c r="I14" s="1">
+        <v>1</v>
+      </c>
+      <c r="J14" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="J14" s="1">
+      <c r="K14" s="1">
         <v>9</v>
       </c>
-      <c r="K14" s="1" t="s">
+      <c r="L14" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="L14" s="1">
-        <v>1</v>
-      </c>
       <c r="M14" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N14" s="1">
         <v>0</v>
       </c>
       <c r="O14" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P14" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q14" s="1">
         <v>0</v>
       </c>
       <c r="R14" s="1">
+        <v>0</v>
+      </c>
+      <c r="S14" s="1">
         <v>0.25</v>
       </c>
-      <c r="S14" s="1">
-        <v>1</v>
-      </c>
       <c r="T14" s="1">
         <v>1</v>
       </c>
@@ -2180,8 +2259,8 @@
       <c r="W14" s="1">
         <v>1</v>
       </c>
-      <c r="X14" s="1" t="s">
-        <v>38</v>
+      <c r="X14" s="1">
+        <v>1</v>
       </c>
       <c r="Y14" s="1" t="s">
         <v>38</v>
@@ -2198,11 +2277,14 @@
       <c r="AC14" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AD14" s="5" t="s">
+      <c r="AD14" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE14" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A15" t="str">
         <f t="shared" si="0"/>
         <v>urine_hat_1.9ml_6_10_years_core</v>
@@ -2215,53 +2297,53 @@
         <v>7</v>
       </c>
       <c r="D15" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="F15" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G15" s="1">
+      <c r="H15" s="1">
         <v>3</v>
       </c>
-      <c r="H15" s="1">
-        <v>1</v>
-      </c>
-      <c r="I15" s="1" t="s">
+      <c r="I15" s="1">
+        <v>1</v>
+      </c>
+      <c r="J15" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="J15" s="1">
+      <c r="K15" s="1">
         <v>10</v>
       </c>
-      <c r="K15" s="1" t="s">
+      <c r="L15" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="L15" s="1">
-        <v>1</v>
-      </c>
       <c r="M15" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N15" s="1">
         <v>0</v>
       </c>
       <c r="O15" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P15" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q15" s="1">
         <v>0</v>
       </c>
       <c r="R15" s="1">
+        <v>0</v>
+      </c>
+      <c r="S15" s="1">
         <v>0.25</v>
       </c>
-      <c r="S15" s="1">
-        <v>1</v>
-      </c>
       <c r="T15" s="1">
         <v>1</v>
       </c>
@@ -2274,8 +2356,8 @@
       <c r="W15" s="1">
         <v>1</v>
       </c>
-      <c r="X15" s="1" t="s">
-        <v>38</v>
+      <c r="X15" s="1">
+        <v>1</v>
       </c>
       <c r="Y15" s="1" t="s">
         <v>38</v>
@@ -2292,11 +2374,14 @@
       <c r="AC15" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AD15" s="5" t="s">
+      <c r="AD15" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE15" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A16" t="str">
         <f t="shared" si="0"/>
         <v>whole_blood_child_1.9ml_6_10_years_core</v>
@@ -2309,53 +2394,53 @@
         <v>2</v>
       </c>
       <c r="D16" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="F16" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G16" s="1">
+      <c r="H16" s="1">
         <v>6</v>
       </c>
-      <c r="H16" s="1">
-        <v>1</v>
-      </c>
-      <c r="I16" s="1" t="s">
+      <c r="I16" s="1">
+        <v>1</v>
+      </c>
+      <c r="J16" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="J16" s="1">
+      <c r="K16" s="1">
         <v>10</v>
       </c>
-      <c r="K16" s="1" t="s">
+      <c r="L16" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="L16" s="1">
-        <v>1</v>
-      </c>
       <c r="M16" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N16" s="1">
         <v>0</v>
       </c>
       <c r="O16" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P16" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q16" s="1">
         <v>0</v>
       </c>
       <c r="R16" s="1">
+        <v>0</v>
+      </c>
+      <c r="S16" s="1">
         <v>0.25</v>
       </c>
-      <c r="S16" s="1">
-        <v>1</v>
-      </c>
       <c r="T16" s="1">
         <v>1</v>
       </c>
@@ -2368,8 +2453,8 @@
       <c r="W16" s="1">
         <v>1</v>
       </c>
-      <c r="X16" s="1" t="s">
-        <v>38</v>
+      <c r="X16" s="1">
+        <v>1</v>
       </c>
       <c r="Y16" s="1" t="s">
         <v>38</v>
@@ -2386,11 +2471,14 @@
       <c r="AC16" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AD16" s="5" t="s">
+      <c r="AD16" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE16" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A17" t="str">
         <f t="shared" si="0"/>
         <v>whole_blood_child_1ml_6_10_years_core</v>
@@ -2403,53 +2491,53 @@
         <v>2</v>
       </c>
       <c r="D17" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="F17" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="G17" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G17" s="1">
+      <c r="H17" s="1">
         <v>10</v>
       </c>
-      <c r="H17" s="1">
+      <c r="I17" s="1">
         <v>0.9</v>
       </c>
-      <c r="I17" s="1" t="s">
+      <c r="J17" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="J17" s="1">
+      <c r="K17" s="1">
         <v>10</v>
       </c>
-      <c r="K17" s="1" t="s">
+      <c r="L17" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="L17" s="1">
-        <v>1</v>
-      </c>
       <c r="M17" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N17" s="1">
         <v>0</v>
       </c>
       <c r="O17" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P17" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q17" s="1">
         <v>0</v>
       </c>
       <c r="R17" s="1">
+        <v>0</v>
+      </c>
+      <c r="S17" s="1">
         <v>0.25</v>
       </c>
-      <c r="S17" s="1">
-        <v>1</v>
-      </c>
       <c r="T17" s="1">
         <v>1</v>
       </c>
@@ -2462,8 +2550,8 @@
       <c r="W17" s="1">
         <v>1</v>
       </c>
-      <c r="X17" s="1" t="s">
-        <v>38</v>
+      <c r="X17" s="1">
+        <v>1</v>
       </c>
       <c r="Y17" s="1" t="s">
         <v>38</v>
@@ -2480,11 +2568,14 @@
       <c r="AC17" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AD17" s="5" t="s">
+      <c r="AD17" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE17" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="18" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A18" t="str">
         <f t="shared" si="0"/>
         <v>urine_cup_current_partner_1.9ml_6_11_months_preconception</v>
@@ -2497,34 +2588,34 @@
         <v>6</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="F18" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="G18" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G18" s="1">
+      <c r="H18" s="1">
         <v>3</v>
       </c>
-      <c r="H18" s="1">
-        <v>1</v>
-      </c>
-      <c r="I18" s="1" t="s">
+      <c r="I18" s="1">
+        <v>1</v>
+      </c>
+      <c r="J18" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J18" s="1">
+      <c r="K18" s="1">
         <v>5</v>
       </c>
-      <c r="K18" s="1" t="s">
+      <c r="L18" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="L18" s="1">
-        <v>0</v>
-      </c>
       <c r="M18" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N18" s="1">
         <v>1</v>
@@ -2539,11 +2630,11 @@
         <v>1</v>
       </c>
       <c r="R18" s="1">
+        <v>1</v>
+      </c>
+      <c r="S18" s="1">
         <v>0.25</v>
       </c>
-      <c r="S18" s="1">
-        <v>1</v>
-      </c>
       <c r="T18" s="1">
         <v>1</v>
       </c>
@@ -2556,8 +2647,8 @@
       <c r="W18" s="1">
         <v>1</v>
       </c>
-      <c r="X18" s="1" t="s">
-        <v>38</v>
+      <c r="X18" s="1">
+        <v>1</v>
       </c>
       <c r="Y18" s="1" t="s">
         <v>38</v>
@@ -2574,11 +2665,14 @@
       <c r="AC18" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AD18" s="5" t="s">
+      <c r="AD18" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE18" s="5" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="19" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A19" t="str">
         <f t="shared" si="0"/>
         <v>urine_cup_maternal_1.9ml_6_11_months_preconception</v>
@@ -2591,32 +2685,32 @@
         <v>5</v>
       </c>
       <c r="D19" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="F19" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="G19" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G19" s="1">
+      <c r="H19" s="1">
         <v>3</v>
       </c>
-      <c r="H19" s="1">
-        <v>1</v>
-      </c>
-      <c r="I19" s="1" t="s">
+      <c r="I19" s="1">
+        <v>1</v>
+      </c>
+      <c r="J19" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J19" s="1">
+      <c r="K19" s="1">
         <v>5</v>
       </c>
-      <c r="K19" s="1" t="s">
+      <c r="L19" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="L19" s="1">
-        <v>1</v>
-      </c>
       <c r="M19" s="1">
         <v>1</v>
       </c>
@@ -2633,11 +2727,11 @@
         <v>1</v>
       </c>
       <c r="R19" s="1">
+        <v>1</v>
+      </c>
+      <c r="S19" s="1">
         <v>0.25</v>
       </c>
-      <c r="S19" s="1">
-        <v>1</v>
-      </c>
       <c r="T19" s="1">
         <v>1</v>
       </c>
@@ -2650,8 +2744,8 @@
       <c r="W19" s="1">
         <v>1</v>
       </c>
-      <c r="X19" s="1" t="s">
-        <v>38</v>
+      <c r="X19" s="1">
+        <v>1</v>
       </c>
       <c r="Y19" s="1" t="s">
         <v>38</v>
@@ -2668,11 +2762,14 @@
       <c r="AC19" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AD19" s="5" t="s">
+      <c r="AD19" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE19" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A20" t="str">
         <f t="shared" si="0"/>
         <v>cord_blood_1.9ml_perinatal_core</v>
@@ -2685,32 +2782,32 @@
         <v>1</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>1</v>
+        <v>67</v>
       </c>
       <c r="E20" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F20" s="1" t="s">
+      <c r="G20" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G20" s="1">
+      <c r="H20" s="1">
         <v>6</v>
       </c>
-      <c r="H20" s="1">
-        <v>1</v>
-      </c>
-      <c r="I20" s="1" t="s">
+      <c r="I20" s="1">
+        <v>1</v>
+      </c>
+      <c r="J20" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="J20" s="1">
+      <c r="K20" s="1">
         <v>3</v>
       </c>
-      <c r="K20" s="1" t="s">
+      <c r="L20" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="L20" s="1">
-        <v>1</v>
-      </c>
       <c r="M20" s="1">
         <v>1</v>
       </c>
@@ -2727,11 +2824,11 @@
         <v>1</v>
       </c>
       <c r="R20" s="1">
+        <v>1</v>
+      </c>
+      <c r="S20" s="1">
         <v>0.25</v>
       </c>
-      <c r="S20" s="1">
-        <v>1</v>
-      </c>
       <c r="T20" s="1">
         <v>1</v>
       </c>
@@ -2744,8 +2841,8 @@
       <c r="W20" s="1">
         <v>1</v>
       </c>
-      <c r="X20" s="1" t="s">
-        <v>38</v>
+      <c r="X20" s="1">
+        <v>1</v>
       </c>
       <c r="Y20" s="1" t="s">
         <v>38</v>
@@ -2762,11 +2859,14 @@
       <c r="AC20" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AD20" s="5" t="s">
+      <c r="AD20" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE20" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="21" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A21" t="str">
         <f t="shared" si="0"/>
         <v>cord_blood_1ml_perinatal_core</v>
@@ -2779,32 +2879,32 @@
         <v>1</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>1</v>
+        <v>67</v>
       </c>
       <c r="E21" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="G21" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G21" s="1">
+      <c r="H21" s="1">
         <v>10</v>
       </c>
-      <c r="H21" s="1">
+      <c r="I21" s="1">
         <v>0.9</v>
       </c>
-      <c r="I21" s="1" t="s">
+      <c r="J21" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="J21" s="1">
+      <c r="K21" s="1">
         <v>3</v>
       </c>
-      <c r="K21" s="1" t="s">
+      <c r="L21" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="L21" s="1">
-        <v>1</v>
-      </c>
       <c r="M21" s="1">
         <v>1</v>
       </c>
@@ -2821,11 +2921,11 @@
         <v>1</v>
       </c>
       <c r="R21" s="1">
+        <v>1</v>
+      </c>
+      <c r="S21" s="1">
         <v>0.25</v>
       </c>
-      <c r="S21" s="1">
-        <v>1</v>
-      </c>
       <c r="T21" s="1">
         <v>1</v>
       </c>
@@ -2838,8 +2938,8 @@
       <c r="W21" s="1">
         <v>1</v>
       </c>
-      <c r="X21" s="1" t="s">
-        <v>38</v>
+      <c r="X21" s="1">
+        <v>1</v>
       </c>
       <c r="Y21" s="1" t="s">
         <v>38</v>
@@ -2856,11 +2956,14 @@
       <c r="AC21" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AD21" s="5" t="s">
+      <c r="AD21" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE21" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A22" t="str">
         <f t="shared" si="0"/>
         <v>placenta_1.9ml_perinatal_core</v>
@@ -2873,32 +2976,32 @@
         <v>9</v>
       </c>
       <c r="D22" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E22" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="F22" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F22" s="1" t="s">
+      <c r="G22" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G22" s="1">
+      <c r="H22" s="1">
         <v>16</v>
       </c>
-      <c r="H22" s="1">
+      <c r="I22" s="1">
         <v>0.9</v>
       </c>
-      <c r="I22" s="1" t="s">
+      <c r="J22" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="J22" s="1">
+      <c r="K22" s="1">
         <v>3</v>
       </c>
-      <c r="K22" s="1" t="s">
+      <c r="L22" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="L22" s="1">
-        <v>1</v>
-      </c>
       <c r="M22" s="1">
         <v>1</v>
       </c>
@@ -2915,11 +3018,11 @@
         <v>1</v>
       </c>
       <c r="R22" s="1">
+        <v>1</v>
+      </c>
+      <c r="S22" s="1">
         <v>0.25</v>
       </c>
-      <c r="S22" s="1">
-        <v>1</v>
-      </c>
       <c r="T22" s="1">
         <v>1</v>
       </c>
@@ -2932,8 +3035,8 @@
       <c r="W22" s="1">
         <v>1</v>
       </c>
-      <c r="X22" s="1" t="s">
-        <v>38</v>
+      <c r="X22" s="1">
+        <v>1</v>
       </c>
       <c r="Y22" s="1" t="s">
         <v>38</v>
@@ -2950,11 +3053,14 @@
       <c r="AC22" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AD22" s="4" t="s">
+      <c r="AD22" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE22" s="4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="23" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A23" t="str">
         <f t="shared" si="0"/>
         <v>urine_cup_maternal_1.9ml_preg_early_core</v>
@@ -2967,32 +3073,32 @@
         <v>5</v>
       </c>
       <c r="D23" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E23" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="F23" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F23" s="1" t="s">
+      <c r="G23" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G23" s="1">
+      <c r="H23" s="1">
         <v>3</v>
       </c>
-      <c r="H23" s="1">
-        <v>1</v>
-      </c>
-      <c r="I23" s="1" t="s">
+      <c r="I23" s="1">
+        <v>1</v>
+      </c>
+      <c r="J23" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J23" s="1">
-        <v>1</v>
-      </c>
-      <c r="K23" s="1" t="s">
+      <c r="K23" s="1">
+        <v>1</v>
+      </c>
+      <c r="L23" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="L23" s="1">
-        <v>1</v>
-      </c>
       <c r="M23" s="1">
         <v>1</v>
       </c>
@@ -3009,11 +3115,11 @@
         <v>1</v>
       </c>
       <c r="R23" s="1">
+        <v>1</v>
+      </c>
+      <c r="S23" s="1">
         <v>0.25</v>
       </c>
-      <c r="S23" s="1">
-        <v>1</v>
-      </c>
       <c r="T23" s="1">
         <v>1</v>
       </c>
@@ -3026,8 +3132,8 @@
       <c r="W23" s="1">
         <v>1</v>
       </c>
-      <c r="X23" s="1" t="s">
-        <v>38</v>
+      <c r="X23" s="1">
+        <v>1</v>
       </c>
       <c r="Y23" s="1" t="s">
         <v>38</v>
@@ -3044,11 +3150,14 @@
       <c r="AC23" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AD23" s="5" t="s">
+      <c r="AD23" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE23" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="24" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A24" t="str">
         <f t="shared" si="0"/>
         <v>whole_blood_maternal_1.9ml_preg_early_core</v>
@@ -3061,32 +3170,32 @@
         <v>0</v>
       </c>
       <c r="D24" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E24" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E24" s="1" t="s">
+      <c r="F24" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F24" s="1" t="s">
+      <c r="G24" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G24" s="1">
+      <c r="H24" s="1">
         <v>6</v>
       </c>
-      <c r="H24" s="1">
-        <v>1</v>
-      </c>
-      <c r="I24" s="1" t="s">
+      <c r="I24" s="1">
+        <v>1</v>
+      </c>
+      <c r="J24" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J24" s="1">
-        <v>1</v>
-      </c>
-      <c r="K24" s="1" t="s">
+      <c r="K24" s="1">
+        <v>1</v>
+      </c>
+      <c r="L24" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="L24" s="1">
-        <v>1</v>
-      </c>
       <c r="M24" s="1">
         <v>1</v>
       </c>
@@ -3103,11 +3212,11 @@
         <v>1</v>
       </c>
       <c r="R24" s="1">
+        <v>1</v>
+      </c>
+      <c r="S24" s="1">
         <v>0.25</v>
       </c>
-      <c r="S24" s="1">
-        <v>1</v>
-      </c>
       <c r="T24" s="1">
         <v>1</v>
       </c>
@@ -3120,8 +3229,8 @@
       <c r="W24" s="1">
         <v>1</v>
       </c>
-      <c r="X24" s="1" t="s">
-        <v>38</v>
+      <c r="X24" s="1">
+        <v>1</v>
       </c>
       <c r="Y24" s="1" t="s">
         <v>38</v>
@@ -3138,11 +3247,14 @@
       <c r="AC24" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AD24" s="5" t="s">
+      <c r="AD24" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE24" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="25" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A25" t="str">
         <f t="shared" si="0"/>
         <v>whole_blood_maternal_1ml_preg_early_core</v>
@@ -3155,32 +3267,32 @@
         <v>0</v>
       </c>
       <c r="D25" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E25" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E25" s="1" t="s">
+      <c r="F25" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F25" s="1" t="s">
+      <c r="G25" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G25" s="1">
+      <c r="H25" s="1">
         <v>10</v>
       </c>
-      <c r="H25" s="1">
+      <c r="I25" s="1">
         <v>0.9</v>
       </c>
-      <c r="I25" s="1" t="s">
+      <c r="J25" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J25" s="1">
-        <v>1</v>
-      </c>
-      <c r="K25" s="1" t="s">
+      <c r="K25" s="1">
+        <v>1</v>
+      </c>
+      <c r="L25" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="L25" s="1">
-        <v>1</v>
-      </c>
       <c r="M25" s="1">
         <v>1</v>
       </c>
@@ -3197,11 +3309,11 @@
         <v>1</v>
       </c>
       <c r="R25" s="1">
+        <v>1</v>
+      </c>
+      <c r="S25" s="1">
         <v>0.25</v>
       </c>
-      <c r="S25" s="1">
-        <v>1</v>
-      </c>
       <c r="T25" s="1">
         <v>1</v>
       </c>
@@ -3214,8 +3326,8 @@
       <c r="W25" s="1">
         <v>1</v>
       </c>
-      <c r="X25" s="1" t="s">
-        <v>38</v>
+      <c r="X25" s="1">
+        <v>1</v>
       </c>
       <c r="Y25" s="1" t="s">
         <v>38</v>
@@ -3232,11 +3344,14 @@
       <c r="AC25" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AD25" s="5" t="s">
+      <c r="AD25" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE25" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="26" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A26" t="str">
         <f t="shared" si="0"/>
         <v>urine_cup_maternal_1.9ml_preg_third_tri_core</v>
@@ -3249,32 +3364,32 @@
         <v>5</v>
       </c>
       <c r="D26" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E26" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E26" s="1" t="s">
+      <c r="F26" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F26" s="1" t="s">
+      <c r="G26" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G26" s="1">
+      <c r="H26" s="1">
         <v>3</v>
       </c>
-      <c r="H26" s="1">
-        <v>1</v>
-      </c>
-      <c r="I26" s="1" t="s">
+      <c r="I26" s="1">
+        <v>1</v>
+      </c>
+      <c r="J26" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J26" s="1">
+      <c r="K26" s="1">
         <v>2</v>
       </c>
-      <c r="K26" s="1" t="s">
+      <c r="L26" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="L26" s="1">
-        <v>1</v>
-      </c>
       <c r="M26" s="1">
         <v>1</v>
       </c>
@@ -3291,11 +3406,11 @@
         <v>1</v>
       </c>
       <c r="R26" s="1">
+        <v>1</v>
+      </c>
+      <c r="S26" s="1">
         <v>0.25</v>
       </c>
-      <c r="S26" s="1">
-        <v>1</v>
-      </c>
       <c r="T26" s="1">
         <v>1</v>
       </c>
@@ -3308,8 +3423,8 @@
       <c r="W26" s="1">
         <v>1</v>
       </c>
-      <c r="X26" s="1" t="s">
-        <v>38</v>
+      <c r="X26" s="1">
+        <v>1</v>
       </c>
       <c r="Y26" s="1" t="s">
         <v>38</v>
@@ -3326,11 +3441,14 @@
       <c r="AC26" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AD26" s="5" t="s">
+      <c r="AD26" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE26" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="27" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A27" t="str">
         <f t="shared" si="0"/>
         <v>whole_blood_maternal_1.9ml_preg_third_tri_core</v>
@@ -3343,32 +3461,32 @@
         <v>0</v>
       </c>
       <c r="D27" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E27" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E27" s="1" t="s">
+      <c r="F27" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F27" s="1" t="s">
+      <c r="G27" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G27" s="1">
+      <c r="H27" s="1">
         <v>6</v>
       </c>
-      <c r="H27" s="1">
-        <v>1</v>
-      </c>
-      <c r="I27" s="1" t="s">
+      <c r="I27" s="1">
+        <v>1</v>
+      </c>
+      <c r="J27" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J27" s="1">
+      <c r="K27" s="1">
         <v>2</v>
       </c>
-      <c r="K27" s="1" t="s">
+      <c r="L27" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="L27" s="1">
-        <v>1</v>
-      </c>
       <c r="M27" s="1">
         <v>1</v>
       </c>
@@ -3385,11 +3503,11 @@
         <v>1</v>
       </c>
       <c r="R27" s="1">
+        <v>1</v>
+      </c>
+      <c r="S27" s="1">
         <v>0.25</v>
       </c>
-      <c r="S27" s="1">
-        <v>1</v>
-      </c>
       <c r="T27" s="1">
         <v>1</v>
       </c>
@@ -3402,8 +3520,8 @@
       <c r="W27" s="1">
         <v>1</v>
       </c>
-      <c r="X27" s="1" t="s">
-        <v>38</v>
+      <c r="X27" s="1">
+        <v>1</v>
       </c>
       <c r="Y27" s="1" t="s">
         <v>38</v>
@@ -3420,11 +3538,14 @@
       <c r="AC27" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AD27" s="5" t="s">
+      <c r="AD27" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE27" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="28" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A28" t="str">
         <f t="shared" si="0"/>
         <v>whole_blood_maternal_1ml_preg_third_tri_core</v>
@@ -3437,32 +3558,32 @@
         <v>0</v>
       </c>
       <c r="D28" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E28" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E28" s="1" t="s">
+      <c r="F28" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="G28" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G28" s="1">
+      <c r="H28" s="1">
         <v>10</v>
       </c>
-      <c r="H28" s="1">
+      <c r="I28" s="1">
         <v>0.9</v>
       </c>
-      <c r="I28" s="1" t="s">
+      <c r="J28" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J28" s="1">
+      <c r="K28" s="1">
         <v>2</v>
       </c>
-      <c r="K28" s="1" t="s">
+      <c r="L28" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="L28" s="1">
-        <v>1</v>
-      </c>
       <c r="M28" s="1">
         <v>1</v>
       </c>
@@ -3479,11 +3600,11 @@
         <v>1</v>
       </c>
       <c r="R28" s="1">
+        <v>1</v>
+      </c>
+      <c r="S28" s="1">
         <v>0.25</v>
       </c>
-      <c r="S28" s="1">
-        <v>1</v>
-      </c>
       <c r="T28" s="1">
         <v>1</v>
       </c>
@@ -3496,8 +3617,8 @@
       <c r="W28" s="1">
         <v>1</v>
       </c>
-      <c r="X28" s="1" t="s">
-        <v>38</v>
+      <c r="X28" s="1">
+        <v>1</v>
       </c>
       <c r="Y28" s="1" t="s">
         <v>38</v>
@@ -3514,101 +3635,104 @@
       <c r="AC28" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AD28" s="4" t="s">
+      <c r="AD28" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE28" s="4" t="s">
         <v>38</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AD28">
-    <sortCondition ref="AC1:AC28"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AE28">
+    <sortCondition ref="AD1:AD28"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="D1:E1048576">
+  <conditionalFormatting sqref="E1:F1048576">
     <cfRule type="containsText" dxfId="23" priority="13" operator="containsText" text="placenta">
-      <formula>NOT(ISERROR(SEARCH("placenta",D1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("placenta",E1)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="22" priority="14" operator="containsText" text="urine">
-      <formula>NOT(ISERROR(SEARCH("urine",D1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("urine",E1)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="21" priority="15" operator="containsText" text="cord_blood">
-      <formula>NOT(ISERROR(SEARCH("cord_blood",D1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("cord_blood",E1)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="20" priority="16" operator="containsText" text="whole_blood">
-      <formula>NOT(ISERROR(SEARCH("whole_blood",D1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("whole_blood",E1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E1:E1048576 I7:J8 I15:J24">
+  <conditionalFormatting sqref="F1:F1048576 J7:K8 J15:K24">
     <cfRule type="containsText" dxfId="19" priority="22" operator="containsText" text="partner">
-      <formula>NOT(ISERROR(SEARCH("partner",E1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("partner",F1)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="18" priority="23" operator="containsText" text="child">
-      <formula>NOT(ISERROR(SEARCH("child",E1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("child",F1)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="17" priority="24" operator="containsText" text="maternal">
-      <formula>NOT(ISERROR(SEARCH("maternal",E1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("maternal",F1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F1:F1048576">
+  <conditionalFormatting sqref="G1:G1048576">
     <cfRule type="containsText" dxfId="16" priority="17" operator="containsText" text="1.9ml">
-      <formula>NOT(ISERROR(SEARCH("1.9ml",F1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("1.9ml",G1)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="15" priority="18" operator="containsText" text="1ml">
-      <formula>NOT(ISERROR(SEARCH("1ml",F1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("1ml",G1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I1:I1048576">
+  <conditionalFormatting sqref="J1:J1048576">
     <cfRule type="containsText" dxfId="14" priority="2" operator="containsText" text="11_17_years">
-      <formula>NOT(ISERROR(SEARCH("11_17_years",I1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("11_17_years",J1)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="13" priority="3" operator="containsText" text="6_10_years">
-      <formula>NOT(ISERROR(SEARCH("6_10_years",I1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("6_10_years",J1)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="12" priority="4" operator="containsText" text="perinatal">
-      <formula>NOT(ISERROR(SEARCH("perinatal",I1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("perinatal",J1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I1:J1048576">
+  <conditionalFormatting sqref="J1:K1048576">
     <cfRule type="containsText" dxfId="11" priority="5" operator="containsText" text="preg_third_tri">
-      <formula>NOT(ISERROR(SEARCH("preg_third_tri",I1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("preg_third_tri",J1)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="10" priority="6" operator="containsText" text="preg_early">
-      <formula>NOT(ISERROR(SEARCH("preg_early",I1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("preg_early",J1)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="9" priority="7" operator="containsText" text="24_35_months">
-      <formula>NOT(ISERROR(SEARCH("24_35_months",I1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("24_35_months",J1)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="8" priority="8" operator="containsText" text="12_23_months">
-      <formula>NOT(ISERROR(SEARCH("12_23_months",I1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("12_23_months",J1)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="7" priority="9" operator="containsText" text="6_11_months">
-      <formula>NOT(ISERROR(SEARCH("6_11_months",I1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("6_11_months",J1)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="6" priority="10" operator="containsText" text="0_5_months">
-      <formula>NOT(ISERROR(SEARCH("0_5_months",I1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("0_5_months",J1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K1:K1048576">
+  <conditionalFormatting sqref="L1:L1048576">
     <cfRule type="containsText" dxfId="5" priority="19" operator="containsText" text="preconception">
-      <formula>NOT(ISERROR(SEARCH("preconception",K1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("preconception",L1)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="4" priority="20" operator="containsText" text="specialized">
-      <formula>NOT(ISERROR(SEARCH("specialized",K1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("specialized",L1)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="3" priority="21" operator="containsText" text="core">
-      <formula>NOT(ISERROR(SEARCH("core",K1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("core",L1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L1:Q1048576">
+  <conditionalFormatting sqref="M1:R1048576">
     <cfRule type="beginsWith" dxfId="2" priority="11" operator="beginsWith" text="0">
-      <formula>LEFT(L1,LEN("0"))="0"</formula>
+      <formula>LEFT(M1,LEN("0"))="0"</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="1" priority="12" operator="containsText" text="1">
-      <formula>NOT(ISERROR(SEARCH("1",L1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("1",M1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X1:AC1048576 AD10:AD28">
+  <conditionalFormatting sqref="Y1:AD1048576 AE10:AE28">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="NA">
-      <formula>NOT(ISERROR(SEARCH("NA",X1)))</formula>
+      <formula>NOT(ISERROR(SEARCH("NA",Y1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>